<commit_message>
docs(management): update task checklists and roadmap workbook (T1.1, T2.3)
</commit_message>
<xml_diff>
--- a/docs/management/DEVOPS_QA_ROADMAP.xlsx
+++ b/docs/management/DEVOPS_QA_ROADMAP.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="218">
   <si>
     <t>DebateSpeak AI — DevOps &amp; QA / Fact-Checking Lead WBS</t>
   </si>
@@ -73,96 +73,111 @@
     <t>CRITICAL</t>
   </si>
   <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>T1.2</t>
+  </si>
+  <si>
+    <t>DevOps / Infra</t>
+  </si>
+  <si>
+    <t>Docker Compose setup for local dev (PostgreSQL 16, Redis 7, LiveKit dev) &amp; clean .env.example</t>
+  </si>
+  <si>
+    <t>docker-compose.yml, .env.example</t>
+  </si>
+  <si>
+    <t>T1.6</t>
+  </si>
+  <si>
+    <t>Management</t>
+  </si>
+  <si>
+    <t>Setup Dev Tools, Scrum Process &amp; Incremental Slices specification</t>
+  </si>
+  <si>
+    <t>docs/management/DEV_TOOLS_AND_PROCESS.md</t>
+  </si>
+  <si>
+    <t>MAJOR</t>
+  </si>
+  <si>
+    <t>T1.8</t>
+  </si>
+  <si>
+    <t>QA / Testing</t>
+  </si>
+  <si>
+    <t>Draft comprehensive QA &amp; Testing Plan (Unit, Integration, Audio chaos, Golden sets)</t>
+  </si>
+  <si>
+    <t>docs/testing/TESTING_PLAN.md</t>
+  </si>
+  <si>
+    <t>R3 (Khoa)</t>
+  </si>
+  <si>
+    <t>T1.9</t>
+  </si>
+  <si>
+    <t>Academic / LaTeX</t>
+  </si>
+  <si>
+    <t>Configure latexmk academic report compilation pipeline &amp; compile submission PDF</t>
+  </si>
+  <si>
+    <t>report/report.tex, report/build/report.pdf</t>
+  </si>
+  <si>
+    <t>R1 (Triết)</t>
+  </si>
+  <si>
+    <t>T2.1</t>
+  </si>
+  <si>
+    <t>Sprint 2 (PA2)</t>
+  </si>
+  <si>
+    <t>Author Project Plan: Goals, deliverables, risks, 5-sprint schedule, build plan</t>
+  </si>
+  <si>
+    <t>docs/pa2/PROJECT_PLAN.md</t>
+  </si>
+  <si>
     <t>In Progress</t>
   </si>
   <si>
-    <t>T1.2</t>
-  </si>
-  <si>
-    <t>DevOps / Infra</t>
-  </si>
-  <si>
-    <t>Docker Compose setup for local dev (PostgreSQL 16, Redis 7, LiveKit dev) &amp; clean .env.example</t>
-  </si>
-  <si>
-    <t>docker-compose.yml, .env.example</t>
-  </si>
-  <si>
-    <t>Done</t>
-  </si>
-  <si>
-    <t>T1.6</t>
-  </si>
-  <si>
-    <t>Management</t>
-  </si>
-  <si>
-    <t>Setup Dev Tools, Scrum Process &amp; Incremental Slices specification</t>
-  </si>
-  <si>
-    <t>docs/management/DEV_TOOLS_AND_PROCESS.md</t>
-  </si>
-  <si>
-    <t>MAJOR</t>
-  </si>
-  <si>
-    <t>T1.8</t>
-  </si>
-  <si>
-    <t>QA / Testing</t>
-  </si>
-  <si>
-    <t>Draft comprehensive QA &amp; Testing Plan (Unit, Integration, Audio chaos, Golden sets)</t>
-  </si>
-  <si>
-    <t>docs/testing/TESTING_PLAN.md</t>
-  </si>
-  <si>
-    <t>R3 (Khoa)</t>
-  </si>
-  <si>
-    <t>T1.9</t>
-  </si>
-  <si>
-    <t>Academic / LaTeX</t>
-  </si>
-  <si>
-    <t>Configure latexmk academic report compilation pipeline &amp; compile submission PDF</t>
-  </si>
-  <si>
-    <t>report/report.tex, report/build/report.pdf</t>
-  </si>
-  <si>
-    <t>R1 (Triết)</t>
-  </si>
-  <si>
-    <t>T2.1</t>
-  </si>
-  <si>
-    <t>Sprint 2 (PA2)</t>
-  </si>
-  <si>
-    <t>Author Project Plan: Goals, deliverables, risks, 5-sprint schedule, build plan</t>
-  </si>
-  <si>
-    <t>docs/pa2/PROJECT_PLAN.md</t>
+    <t>T2.3</t>
+  </si>
+  <si>
+    <t>SDD / Spec Kit</t>
+  </si>
+  <si>
+    <t>Spec Kit Initialization in /src: constitution.md and initial spec artifacts</t>
+  </si>
+  <si>
+    <t>src/constitution.md, .specify/</t>
+  </si>
+  <si>
+    <t>R4 (Tuấn)</t>
+  </si>
+  <si>
+    <t>T2.R</t>
+  </si>
+  <si>
+    <t>QA / Review</t>
+  </si>
+  <si>
+    <t>Verify Backend Build 1: PostgreSQL migrations, Argon2id auth, JWT rotation, and room lobby endpoints</t>
+  </si>
+  <si>
+    <t>api/tests/unit/test_auth.py</t>
   </si>
   <si>
     <t>Planned</t>
   </si>
   <si>
-    <t>T2.R</t>
-  </si>
-  <si>
-    <t>QA / Review</t>
-  </si>
-  <si>
-    <t>Verify Backend Build 1: PostgreSQL migrations, Argon2id auth, JWT rotation, and room lobby endpoints</t>
-  </si>
-  <si>
-    <t>api/tests/unit/test_auth.py</t>
-  </si>
-  <si>
     <t>T3.1</t>
   </si>
   <si>
@@ -241,9 +256,6 @@
     <t>docs/pa5/DEFECT_MATRIX.md</t>
   </si>
   <si>
-    <t>R4 (Tuấn)</t>
-  </si>
-  <si>
     <t>T5.3</t>
   </si>
   <si>
@@ -349,9 +361,6 @@
     <t>Tài (R2), Triết (R1)</t>
   </si>
   <si>
-    <t>15 mins</t>
-  </si>
-  <si>
     <t>Step 4</t>
   </si>
   <si>
@@ -367,22 +376,16 @@
     <t>All coders</t>
   </si>
   <si>
-    <t>30 mins</t>
-  </si>
-  <si>
     <t>Step 5</t>
   </si>
   <si>
     <t>GitHub Actions CI Pipeline (.github/workflows/ci.yml)</t>
   </si>
   <si>
-    <t>Automates linting, security audits (pip-audit), tests, and latexmk build</t>
+    <t>Automates linting, security audits, tests, and latexmk build</t>
   </si>
   <si>
     <t>All PRs</t>
-  </si>
-  <si>
-    <t>1 hour</t>
   </si>
   <si>
     <t>Step 6</t>
@@ -728,14 +731,6 @@
     <font>
       <b/>
       <sz val="10"/>
-      <color rgb="FF92400E"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
       <color rgb="FF065F46"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -744,6 +739,14 @@
     <font>
       <sz val="10"/>
       <color rgb="FFB45309"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF92400E"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -777,13 +780,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFEF3C7"/>
+        <fgColor rgb="FFD1FAE5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD1FAE5"/>
+        <fgColor rgb="FFFEF3C7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -850,7 +853,7 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1156,7 +1159,7 @@
   <sheetPr>
     <tabColor rgb="FF1E3A8A"/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.7109375" customWidth="1"/>
@@ -1276,25 +1279,25 @@
       <c r="H6" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="9" t="s">
-        <v>23</v>
+      <c r="I6" s="8" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="E7" s="5" t="s">
         <v>26</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>27</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>16</v>
@@ -1302,31 +1305,31 @@
       <c r="G7" s="6">
         <v>3</v>
       </c>
-      <c r="H7" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="I7" s="9" t="s">
-        <v>23</v>
+      <c r="H7" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="E8" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="F8" s="4" t="s">
         <v>32</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>33</v>
       </c>
       <c r="G8" s="6">
         <v>5</v>
@@ -1334,57 +1337,57 @@
       <c r="H8" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="I8" s="9" t="s">
-        <v>23</v>
+      <c r="I8" s="8" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>12</v>
       </c>
       <c r="C9" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="E9" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="F9" s="4" t="s">
         <v>37</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>38</v>
       </c>
       <c r="G9" s="6">
         <v>2</v>
       </c>
-      <c r="H9" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="I9" s="9" t="s">
-        <v>23</v>
+      <c r="H9" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I9" s="8" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="C10" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D10" s="5" t="s">
+      <c r="E10" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="E10" s="5" t="s">
-        <v>42</v>
-      </c>
       <c r="F10" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G10" s="6">
         <v>5</v>
@@ -1392,37 +1395,37 @@
       <c r="H10" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="I10" s="11" t="s">
-        <v>43</v>
+      <c r="I10" s="10" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:9">
       <c r="A11" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B11" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" s="4" t="s">
+      <c r="D11" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="E11" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="F11" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="G11" s="6">
-        <v>2</v>
-      </c>
-      <c r="H11" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="I11" s="11" t="s">
-        <v>43</v>
+        <v>3</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="I11" s="8" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -1430,10 +1433,10 @@
         <v>48</v>
       </c>
       <c r="B12" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>25</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>50</v>
@@ -1442,190 +1445,190 @@
         <v>51</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="G12" s="6">
-        <v>3</v>
-      </c>
-      <c r="H12" s="10" t="s">
-        <v>28</v>
+        <v>2</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:9">
       <c r="A13" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G13" s="6">
         <v>3</v>
       </c>
-      <c r="H13" s="7" t="s">
-        <v>17</v>
+      <c r="H13" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:9">
       <c r="A14" s="4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="G14" s="6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H14" s="7" t="s">
         <v>17</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:9">
       <c r="A15" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="G15" s="6">
-        <v>2</v>
-      </c>
-      <c r="H15" s="10" t="s">
-        <v>28</v>
+        <v>5</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:9">
       <c r="A16" s="4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>63</v>
+        <v>24</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="G16" s="6">
-        <v>3</v>
-      </c>
-      <c r="H16" s="7" t="s">
-        <v>17</v>
+        <v>2</v>
+      </c>
+      <c r="H16" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>30</v>
+        <v>68</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G17" s="6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H17" s="7" t="s">
         <v>17</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
     </row>
     <row r="18" spans="1:9">
       <c r="A18" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>74</v>
+        <v>16</v>
       </c>
       <c r="G18" s="6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H18" s="7" t="s">
         <v>17</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -1633,7 +1636,7 @@
         <v>75</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>76</v>
@@ -1645,16 +1648,16 @@
         <v>78</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>16</v>
+        <v>47</v>
       </c>
       <c r="G19" s="6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H19" s="7" t="s">
         <v>17</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -1662,19 +1665,19 @@
         <v>79</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>25</v>
+        <v>80</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>82</v>
+        <v>16</v>
       </c>
       <c r="G20" s="6">
         <v>5</v>
@@ -1683,7 +1686,7 @@
         <v>17</v>
       </c>
       <c r="I20" s="11" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -1691,28 +1694,57 @@
         <v>83</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C21" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D21" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="E21" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="E21" s="5" t="s">
+      <c r="F21" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="F21" s="4" t="s">
-        <v>82</v>
-      </c>
       <c r="G21" s="6">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H21" s="7" t="s">
         <v>17</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>43</v>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="G22" s="6">
+        <v>2</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="I22" s="11" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1742,7 +1774,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1753,7 +1785,7 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="2" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1764,22 +1796,22 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="3" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>10</v>
@@ -1787,68 +1819,68 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="4" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="G5" s="9" t="s">
-        <v>23</v>
+        <v>103</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="4" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="D6" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="E6" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>23</v>
+      <c r="G6" s="8" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="4" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>18</v>
@@ -1856,71 +1888,71 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="4" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="G8" s="11" t="s">
-        <v>43</v>
+        <v>103</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="4" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>15</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="G9" s="11" t="s">
-        <v>43</v>
+        <v>103</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="4" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C10" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="G10" s="10" t="s">
         <v>42</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="G10" s="11" t="s">
-        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1950,7 +1982,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1960,7 +1992,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1970,162 +2002,162 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>141</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="4" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="4" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="4" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="4" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -2156,7 +2188,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2167,7 +2199,7 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2178,36 +2210,36 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D5" s="12">
         <v>0</v>
@@ -2216,21 +2248,21 @@
         <v>0</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D6" s="12">
         <v>0.0043</v>
@@ -2239,21 +2271,21 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="5" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D7" s="12">
         <v>0.00025</v>
@@ -2262,21 +2294,21 @@
         <v>0.0015</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D8" s="12">
         <v>0.00025</v>
@@ -2285,21 +2317,21 @@
         <v>0.0016</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="5" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D9" s="12">
         <v>0.00025</v>
@@ -2308,21 +2340,21 @@
         <v>0.001</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D10" s="12">
         <v>0.00025</v>
@@ -2331,21 +2363,21 @@
         <v>0.002</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="5" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D11" s="12">
         <v>0.001</v>
@@ -2354,21 +2386,21 @@
         <v>0.016</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D12" s="12">
         <v>10</v>
@@ -2377,15 +2409,15 @@
         <v>0.02</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="3" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -2394,10 +2426,10 @@
         <f>SUM(E5:E12)</f>
         <v>0</v>
       </c>
-      <c r="F13" s="9" t="s">
-        <v>216</v>
-      </c>
-      <c r="G13" s="9"/>
+      <c r="F13" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="G13" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>